<commit_message>
Complete POC-03 registration design
</commit_message>
<xml_diff>
--- a/docs/sharepoint_schema_import_template.xlsx
+++ b/docs/sharepoint_schema_import_template.xlsx
@@ -2,9 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="R559b25dcb8f944e0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Language catalogue" sheetId="2" r:id="Ra4088d417f074593"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participants" sheetId="3" r:id="R8ed2d9bcff1b4f12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" r:id="Rc84899b7a1a34c22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Language catalogue" sheetId="2" r:id="Rb5ce50091e2a416f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Participants" sheetId="3" r:id="Rc53935bde53e46ae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Time zone catalogue" sheetId="4" r:id="Rab968d0debfb4258"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -15,7 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="5">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -44,8 +45,42 @@
       <x:color rgb="FF9C0006"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF000000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FFC00000"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF1F4E78"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="14"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -67,6 +102,36 @@
         <x:fgColor rgb="FFFCE4D6"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="13">
     <x:border/>
@@ -221,7 +286,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="35">
+  <x:cellXfs count="65">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -305,11 +370,123 @@
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1">
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -325,17 +502,52 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="ParticipantsImport" displayName="ParticipantsImport" ref="A4:I5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:tableColumns count="9">
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="5" name="ParticipantsImport" displayName="ParticipantsImport" ref="A4:H5" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="8">
     <x:tableColumn id="1" name="Title"/>
     <x:tableColumn id="2" name="Participant account"/>
     <x:tableColumn id="3" name="Teach languages"/>
     <x:tableColumn id="4" name="Learn languages"/>
-    <x:tableColumn id="5" name="Location"/>
-    <x:tableColumn id="6" name="Time zone"/>
-    <x:tableColumn id="7" name="Learning focus"/>
-    <x:tableColumn id="8" name="Comments"/>
-    <x:tableColumn id="9" name="Status"/>
+    <x:tableColumn id="5" name="Time zone"/>
+    <x:tableColumn id="6" name="Learning focus"/>
+    <x:tableColumn id="7" name="Comments"/>
+    <x:tableColumn id="8" name="Status"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="TimeZoneCatalogueImport" displayName="TimeZoneCatalogueImport" ref="A1:D11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="Time zone catalogue import template"/>
+    <x:tableColumn id="2" name="Column2"/>
+    <x:tableColumn id="3" name="Column3"/>
+    <x:tableColumn id="4" name="Column4"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="4" name="TimeZoneCatalogueImport" displayName="TimeZoneCatalogueImport" ref="A1:D11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="Time zone catalogue import template"/>
+    <x:tableColumn id="2" name="Column2"/>
+    <x:tableColumn id="3" name="Column3"/>
+    <x:tableColumn id="4" name="Column4"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="TimeZoneCatalogueImport" displayName="TimeZoneCatalogueImport" ref="A1:D11" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="4">
+    <x:tableColumn id="1" name="Time zone catalogue import template"/>
+    <x:tableColumn id="2" name="Column2"/>
+    <x:tableColumn id="3" name="Column3"/>
+    <x:tableColumn id="4" name="Column4"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
@@ -547,7 +759,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="4" t="str">
-        <x:v>Generated from SharePoint schema version 2. The workbook creates headings and import guidance; SharePoint field types still need checking after Excel import.</x:v>
+        <x:v>Generated from SharePoint schema version 3. The workbook creates headings and import guidance; SharePoint field types still need checking after Excel import.</x:v>
       </x:c>
       <x:c r="B2" s="4"/>
       <x:c r="C2" s="4"/>
@@ -582,7 +794,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="15" t="str">
-        <x:v>Import the Participants sheet, or create it from the existing list if one already exists.</x:v>
+        <x:v>Import the Time zone catalogue sheet, then import the Participants sheet or create it from the existing list if one already exists.</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -590,7 +802,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B8" s="15" t="str">
-        <x:v>After import, configure Person, Lookup, Location, Choice, and Yes/No fields using the field notes on each sheet.</x:v>
+        <x:v>After import, configure Person, Lookup, Choice, Yes/No, and optional text fields using the field notes on each sheet.</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -606,7 +818,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B10" s="15" t="str">
-        <x:v>Set Status choices to Active and Needs review. Location is required; Time zone can be filled by the flow later.</x:v>
+        <x:v>Set Time zone as a required single-value Lookup to Time zone catalogue → Title. Location/city and culture-interest fields are deferred. Set Status choices to Active and Needs review.</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -755,7 +967,7 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbea8e7a2a4d146da"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd63ad3d980f245de"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -790,7 +1002,7 @@
     </x:row>
     <x:row r="2">
       <x:c r="A2" s="24" t="str">
-        <x:v>The highlighted sample row keeps the Excel table valid. Delete it after importing the list.</x:v>
+        <x:v>Import this sheet to create the column headings. Delete the highlighted sample row after importing.</x:v>
       </x:c>
       <x:c r="B2" s="24"/>
       <x:c r="C2" s="24"/>
@@ -826,33 +1038,43 @@
         <x:v>Learn languages</x:v>
       </x:c>
       <x:c r="E4" s="19" t="str">
-        <x:v>Location</x:v>
+        <x:v>Time zone</x:v>
       </x:c>
       <x:c r="F4" s="19" t="str">
-        <x:v>Time zone</x:v>
+        <x:v>Learning focus</x:v>
       </x:c>
       <x:c r="G4" s="19" t="str">
-        <x:v>Learning focus</x:v>
+        <x:v>Comments</x:v>
       </x:c>
       <x:c r="H4" s="19" t="str">
-        <x:v>Comments</x:v>
-      </x:c>
-      <x:c r="I4" s="14" t="str">
         <x:v>Status</x:v>
       </x:c>
+      <x:c r="I4" s="14"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="25" t="str">
         <x:v>DELETE THIS SAMPLE ROW</x:v>
       </x:c>
-      <x:c r="B5" s="25" t="str"/>
-      <x:c r="C5" s="25" t="str"/>
-      <x:c r="D5" s="25" t="str"/>
-      <x:c r="E5" s="25" t="str"/>
-      <x:c r="F5" s="25" t="str"/>
-      <x:c r="G5" s="25" t="str"/>
-      <x:c r="H5" s="25" t="str"/>
-      <x:c r="I5" s="25" t="str"/>
+      <x:c r="B5" s="25"/>
+      <x:c r="C5" s="25"/>
+      <x:c r="D5" s="25"/>
+      <x:c r="E5" s="25"/>
+      <x:c r="F5" s="25"/>
+      <x:c r="G5" s="25"/>
+      <x:c r="H5" s="25" t="str">
+        <x:v>Needs review</x:v>
+      </x:c>
+      <x:c r="I5" s="25"/>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6"/>
+      <x:c r="B6"/>
+      <x:c r="C6"/>
+      <x:c r="D6"/>
+      <x:c r="E6"/>
+      <x:c r="F6"/>
+      <x:c r="G6"/>
+      <x:c r="H6"/>
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="26" t="str">
@@ -867,6 +1089,10 @@
       <x:c r="D7" s="28" t="str">
         <x:v>Import note</x:v>
       </x:c>
+      <x:c r="E7"/>
+      <x:c r="F7"/>
+      <x:c r="G7"/>
+      <x:c r="H7"/>
     </x:row>
     <x:row r="8">
       <x:c r="A8" s="29" t="str">
@@ -879,22 +1105,30 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="D8" s="31" t="str">
-        <x:v>Imported from the Excel heading.</x:v>
-      </x:c>
+        <x:v>System text; hide from the participant form.</x:v>
+      </x:c>
+      <x:c r="E8"/>
+      <x:c r="F8"/>
+      <x:c r="G8"/>
+      <x:c r="H8"/>
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="29" t="str">
         <x:v>Participant account</x:v>
       </x:c>
       <x:c r="B9" s="30" t="str">
-        <x:v>User</x:v>
+        <x:v>Person</x:v>
       </x:c>
       <x:c r="C9" s="30" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="D9" s="31" t="str">
-        <x:v>Configure as Person after import.</x:v>
-      </x:c>
+        <x:v>One person; set unique values and index this column.</x:v>
+      </x:c>
+      <x:c r="E9"/>
+      <x:c r="F9"/>
+      <x:c r="G9"/>
+      <x:c r="H9"/>
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="29" t="str">
@@ -907,8 +1141,12 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="D10" s="31" t="str">
-        <x:v>Configure as multi-select Lookup to Language catalogue.</x:v>
-      </x:c>
+        <x:v>Multiple-value Lookup to Language catalogue → Title.</x:v>
+      </x:c>
+      <x:c r="E10"/>
+      <x:c r="F10"/>
+      <x:c r="G10"/>
+      <x:c r="H10"/>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="29" t="str">
@@ -921,78 +1159,94 @@
         <x:v>No</x:v>
       </x:c>
       <x:c r="D11" s="31" t="str">
-        <x:v>Configure as multi-select Lookup to Language catalogue.</x:v>
-      </x:c>
+        <x:v>Multiple-value Lookup to Language catalogue → Title.</x:v>
+      </x:c>
+      <x:c r="E11"/>
+      <x:c r="F11"/>
+      <x:c r="G11"/>
+      <x:c r="H11"/>
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="29" t="str">
-        <x:v>Location</x:v>
+        <x:v>Time zone</x:v>
       </x:c>
       <x:c r="B12" s="30" t="str">
-        <x:v>Location</x:v>
+        <x:v>Lookup</x:v>
       </x:c>
       <x:c r="C12" s="30" t="str">
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="D12" s="31" t="str">
-        <x:v>Configure as Location after import; provisioning is manual.</x:v>
-      </x:c>
+        <x:v>Single-value Lookup to Time zone catalogue → Title; use active values.</x:v>
+      </x:c>
+      <x:c r="E12"/>
+      <x:c r="F12"/>
+      <x:c r="G12"/>
+      <x:c r="H12"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="29" t="str">
-        <x:v>Time zone</x:v>
+        <x:v>Learning focus</x:v>
       </x:c>
       <x:c r="B13" s="30" t="str">
-        <x:v>Text</x:v>
+        <x:v>Multiple lines</x:v>
       </x:c>
       <x:c r="C13" s="30" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="D13" s="31" t="str">
-        <x:v>Imported from the Excel heading.</x:v>
-      </x:c>
+        <x:v>Optional participant context.</x:v>
+      </x:c>
+      <x:c r="E13"/>
+      <x:c r="F13"/>
+      <x:c r="G13"/>
+      <x:c r="H13"/>
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="29" t="str">
-        <x:v>Learning focus</x:v>
+        <x:v>Comments</x:v>
       </x:c>
       <x:c r="B14" s="30" t="str">
-        <x:v>Note</x:v>
+        <x:v>Multiple lines</x:v>
       </x:c>
       <x:c r="C14" s="30" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="D14" s="31" t="str">
-        <x:v>Imported from the Excel heading.</x:v>
-      </x:c>
+        <x:v>Optional participant context.</x:v>
+      </x:c>
+      <x:c r="E14"/>
+      <x:c r="F14"/>
+      <x:c r="G14"/>
+      <x:c r="H14"/>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="29" t="str">
-        <x:v>Comments</x:v>
+        <x:v>Status</x:v>
       </x:c>
       <x:c r="B15" s="30" t="str">
-        <x:v>Note</x:v>
+        <x:v>Choice</x:v>
       </x:c>
       <x:c r="C15" s="30" t="str">
         <x:v>No</x:v>
       </x:c>
       <x:c r="D15" s="31" t="str">
-        <x:v>Imported from the Excel heading.</x:v>
-      </x:c>
+        <x:v>Flow-managed choices: Active; Needs review. Hide from the participant form.</x:v>
+      </x:c>
+      <x:c r="E15"/>
+      <x:c r="F15"/>
+      <x:c r="G15"/>
+      <x:c r="H15"/>
     </x:row>
     <x:row r="16">
-      <x:c r="A16" s="32" t="str">
-        <x:v>Status</x:v>
-      </x:c>
-      <x:c r="B16" s="33" t="str">
-        <x:v>Choice</x:v>
-      </x:c>
-      <x:c r="C16" s="33" t="str">
-        <x:v>No</x:v>
-      </x:c>
-      <x:c r="D16" s="34" t="str">
-        <x:v>Configure choices: Active, Needs review.</x:v>
-      </x:c>
+      <x:c r="A16" s="32"/>
+      <x:c r="B16" s="33"/>
+      <x:c r="C16" s="33"/>
+      <x:c r="D16" s="34"/>
+      <x:c r="E16"/>
+      <x:c r="F16"/>
+      <x:c r="G16"/>
+      <x:c r="H16"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -1000,7 +1254,149 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd4dbdf8c7ad2455d"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9e0c5cfca5e14b25"/>
+  </x:tableParts>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="24" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="58" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" s="57" t="str">
+        <x:v>Time zone catalogue import template</x:v>
+      </x:c>
+      <x:c r="B1" s="57"/>
+      <x:c r="C1" s="57"/>
+      <x:c r="D1" s="57"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="62" t="str">
+        <x:v>The highlighted sample row keeps the Excel table valid. Delete it after importing the list.</x:v>
+      </x:c>
+      <x:c r="B2" s="62"/>
+      <x:c r="C2" s="62"/>
+      <x:c r="D2" s="62"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="48"/>
+      <x:c r="B3" s="48"/>
+      <x:c r="C3" s="48"/>
+      <x:c r="D3" s="48"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="63" t="str">
+        <x:v>Time zone</x:v>
+      </x:c>
+      <x:c r="B4" s="63" t="str">
+        <x:v>IANA ID</x:v>
+      </x:c>
+      <x:c r="C4" s="63" t="str">
+        <x:v>Windows ID</x:v>
+      </x:c>
+      <x:c r="D4" s="63" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="50" t="str">
+        <x:v>DELETE THIS SAMPLE ROW</x:v>
+      </x:c>
+      <x:c r="B5" s="50"/>
+      <x:c r="C5" s="50"/>
+      <x:c r="D5" s="51" t="b">
+        <x:v>1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="48"/>
+      <x:c r="B6" s="48"/>
+      <x:c r="C6" s="48"/>
+      <x:c r="D6" s="48"/>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="64" t="str">
+        <x:v>Field</x:v>
+      </x:c>
+      <x:c r="B7" s="64" t="str">
+        <x:v>SharePoint type</x:v>
+      </x:c>
+      <x:c r="C7" s="64" t="str">
+        <x:v>Required</x:v>
+      </x:c>
+      <x:c r="D7" s="64" t="str">
+        <x:v>Import note</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="48" t="str">
+        <x:v>Time zone</x:v>
+      </x:c>
+      <x:c r="B8" s="48" t="str">
+        <x:v>Text</x:v>
+      </x:c>
+      <x:c r="C8" s="48" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D8" s="48" t="str">
+        <x:v>Imported from the Excel heading; use as the lookup display column.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="48" t="str">
+        <x:v>IANA ID</x:v>
+      </x:c>
+      <x:c r="B9" s="48" t="str">
+        <x:v>Text</x:v>
+      </x:c>
+      <x:c r="C9" s="48" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="D9" s="48" t="str">
+        <x:v>Set as unique and indexed, for example Europe/Berlin.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="48" t="str">
+        <x:v>Windows ID</x:v>
+      </x:c>
+      <x:c r="B10" s="48" t="str">
+        <x:v>Text</x:v>
+      </x:c>
+      <x:c r="C10" s="48" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D10" s="48" t="str">
+        <x:v>Optional compatibility identifier.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="48" t="str">
+        <x:v>Active</x:v>
+      </x:c>
+      <x:c r="B11" s="48" t="str">
+        <x:v>Boolean</x:v>
+      </x:c>
+      <x:c r="C11" s="48" t="str">
+        <x:v>No</x:v>
+      </x:c>
+      <x:c r="D11" s="48" t="str">
+        <x:v>Configure as Yes/No; default is Yes.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="3">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R56005bd9249143a3"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rcc124ae84a4f499c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re4832b93dca04b30"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>